<commit_message>
Regenerate the workbook template from reviewed styling sources
</commit_message>
<xml_diff>
--- a/src/workbook/FRTB_Template.xlsx
+++ b/src/workbook/FRTB_Template.xlsx
@@ -1825,7 +1825,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="9">
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
@@ -1850,6 +1850,96 @@
         <color rgb="FFBFBFBF"/>
       </right>
       <top style="thin">
+        <color rgb="FFBFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFBFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin">
+        <color rgb="FFBFBFBF"/>
+      </left>
+      <right style="dashed">
+        <color rgb="FFBFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFBFBFBF"/>
+      </top>
+      <bottom style="dashed">
+        <color rgb="FFBFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="dashed">
+        <color rgb="FFBFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFBFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFBFBFBF"/>
+      </top>
+      <bottom style="dashed">
+        <color rgb="FFBFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin">
+        <color rgb="FFBFBFBF"/>
+      </left>
+      <right style="dashed">
+        <color rgb="FFBFBFBF"/>
+      </right>
+      <top style="dashed">
+        <color rgb="FFBFBFBF"/>
+      </top>
+      <bottom style="dashed">
+        <color rgb="FFBFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="dashed">
+        <color rgb="FFBFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFBFBFBF"/>
+      </right>
+      <top style="dashed">
+        <color rgb="FFBFBFBF"/>
+      </top>
+      <bottom style="dashed">
+        <color rgb="FFBFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin">
+        <color rgb="FFBFBFBF"/>
+      </left>
+      <right style="dashed">
+        <color rgb="FFBFBFBF"/>
+      </right>
+      <top style="dashed">
+        <color rgb="FFBFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFBFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="dashed">
+        <color rgb="FFBFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFBFBFBF"/>
+      </right>
+      <top style="dashed">
         <color rgb="FFBFBFBF"/>
       </top>
       <bottom style="thin">
@@ -1883,7 +1973,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="37">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -2006,6 +2096,30 @@
     </xf>
     <xf numFmtId="169" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="1" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="1" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="1" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="1" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="1" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="8" xfId="0" applyFont="true" applyBorder="1" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -2266,58 +2380,58 @@
       <c r="D5" s="8"/>
     </row>
     <row r="6" customFormat="false" ht="33.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C6" s="9" t="s">
+      <c r="C6" s="31" t="s">
         <v>4</v>
       </c>
-      <c r="D6" s="10" t="s">
+      <c r="D6" s="32" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="33.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C7" s="9" t="s">
+      <c r="C7" s="33" t="s">
         <v>6</v>
       </c>
-      <c r="D7" s="10" t="s">
+      <c r="D7" s="34" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="33.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C8" s="9" t="s">
+      <c r="C8" s="33" t="s">
         <v>8</v>
       </c>
-      <c r="D8" s="10" t="s">
+      <c r="D8" s="34" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="33.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C9" s="9" t="s">
+      <c r="C9" s="33" t="s">
         <v>10</v>
       </c>
-      <c r="D9" s="10" t="s">
+      <c r="D9" s="34" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="33.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C10" s="9" t="s">
+      <c r="C10" s="33" t="s">
         <v>12</v>
       </c>
-      <c r="D10" s="10" t="s">
+      <c r="D10" s="34" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="33.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C11" s="9" t="s">
+      <c r="C11" s="33" t="s">
         <v>14</v>
       </c>
-      <c r="D11" s="10" t="s">
+      <c r="D11" s="34" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="33.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C12" s="9" t="s">
+      <c r="C12" s="35" t="s">
         <v>16</v>
       </c>
-      <c r="D12" s="10" t="s">
+      <c r="D12" s="36" t="s">
         <v>17</v>
       </c>
     </row>
@@ -2328,58 +2442,58 @@
       <c r="D14" s="8"/>
     </row>
     <row r="15" customFormat="false" ht="33.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C15" s="9" t="s">
+      <c r="C15" s="31" t="s">
         <v>19</v>
       </c>
-      <c r="D15" s="10" t="s">
+      <c r="D15" s="32" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="33.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C16" s="9" t="s">
+      <c r="C16" s="33" t="s">
         <v>21</v>
       </c>
-      <c r="D16" s="10" t="s">
+      <c r="D16" s="34" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="33.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C17" s="9" t="s">
+      <c r="C17" s="33" t="s">
         <v>23</v>
       </c>
-      <c r="D17" s="10" t="s">
+      <c r="D17" s="34" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="33.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C18" s="9" t="s">
+      <c r="C18" s="33" t="s">
         <v>25</v>
       </c>
-      <c r="D18" s="10" t="s">
+      <c r="D18" s="34" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="33.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C19" s="9" t="s">
+      <c r="C19" s="33" t="s">
         <v>27</v>
       </c>
-      <c r="D19" s="10" t="s">
+      <c r="D19" s="34" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="33.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C20" s="9" t="s">
+      <c r="C20" s="33" t="s">
         <v>29</v>
       </c>
-      <c r="D20" s="10" t="s">
+      <c r="D20" s="34" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="33.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C21" s="9" t="s">
+      <c r="C21" s="35" t="s">
         <v>31</v>
       </c>
-      <c r="D21" s="10" t="s">
+      <c r="D21" s="36" t="s">
         <v>32</v>
       </c>
     </row>
@@ -2390,26 +2504,26 @@
       <c r="D23" s="8"/>
     </row>
     <row r="24" customFormat="false" ht="33.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C24" s="9" t="s">
+      <c r="C24" s="31" t="s">
         <v>34</v>
       </c>
-      <c r="D24" s="10" t="s">
+      <c r="D24" s="32" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="33.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C25" s="9" t="s">
+      <c r="C25" s="33" t="s">
         <v>36</v>
       </c>
-      <c r="D25" s="10" t="s">
+      <c r="D25" s="34" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="33.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C26" s="9" t="s">
+      <c r="C26" s="35" t="s">
         <v>38</v>
       </c>
-      <c r="D26" s="10" t="s">
+      <c r="D26" s="36" t="s">
         <v>39</v>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: cite the paragraph that holds each rule (#116)
Correct MAR references that pointed to the wrong paragraph, checked against the BIS text on 2026-10-27: netting MAR21.4(2); commodity tenors MAR21.13(1); vega maturities MAR21.8(4); DRC floor MAR22.18 and horizon MAR22.15; RRAO MAR23.8(2)(a) and (b); the CORE_DRC step comments; sensitivity definitions MAR21.19-26; and the sources of the framework diagram. The template is rebuilt: eight reference cells change; no parameter value or result changes.

Validated at c73729a: vba_lint 0 problems; build_template and update_expected --check current; REQUIRE_LIBREOFFICE=1 pytest 188 passed, 29 subtests; hosted Repository integrity and LibreOffice reconciliation passed; Codex review found no issues. Not validated: Excel.

Resolves #115
</commit_message>
<xml_diff>
--- a/src/workbook/FRTB_Template.xlsx
+++ b/src/workbook/FRTB_Template.xlsx
@@ -178,7 +178,7 @@
     <t xml:space="preserve">Amounts</t>
   </si>
   <si>
-    <t xml:space="preserve">Sensitivities as defined in MAR21.18-26 (for example GIRR: PV change for 1bp / 0.0001). Vega: vega x implied volatility. Curvature: CVR up and CVR down per risk factor.</t>
+    <t xml:space="preserve">Sensitivities as defined in MAR21.19-26 (for example GIRR: PV change for 1bp / 0.0001). Vega: vega x implied volatility. Curvature: CVR up and CVR down per risk factor.</t>
   </si>
   <si>
     <t xml:space="preserve">DRC</t>
@@ -295,7 +295,7 @@
     <t xml:space="preserve">Delta sensitivities</t>
   </si>
   <si>
-    <t xml:space="preserve">Delta sensitivities in the reporting currency; rows with the same risk factor are netted (MAR21.4(1)).</t>
+    <t xml:space="preserve">Delta sensitivities in the reporting currency; rows with the same risk factor are netted (MAR21.4(2)).</t>
   </si>
   <si>
     <t xml:space="preserve">ID</t>
@@ -1048,13 +1048,13 @@
     <t xml:space="preserve">0,0.25,0.5,1,2,3,5,10,15,20,30</t>
   </si>
   <si>
-    <t xml:space="preserve">MAR21.12(1)</t>
+    <t xml:space="preserve">MAR21.13(1)</t>
   </si>
   <si>
     <t xml:space="preserve">VEGA_MATURITIES</t>
   </si>
   <si>
-    <t xml:space="preserve">MAR21.8(2)</t>
+    <t xml:space="preserve">MAR21.8(4)</t>
   </si>
   <si>
     <t xml:space="preserve">Interest rate parameters</t>
@@ -1471,13 +1471,13 @@
     <t xml:space="preserve">MIN_MATURITY</t>
   </si>
   <si>
-    <t xml:space="preserve">MAR22.17: floor of three months</t>
+    <t xml:space="preserve">MAR22.18: floor of three months</t>
   </si>
   <si>
     <t xml:space="preserve">MAX_MATURITY</t>
   </si>
   <si>
-    <t xml:space="preserve">MAR22.17: one-year capital horizon</t>
+    <t xml:space="preserve">MAR22.15: one-year capital horizon</t>
   </si>
   <si>
     <t xml:space="preserve">[DRC_BUCKETS]  Buckets (MAR22.22)</t>
@@ -1501,10 +1501,10 @@
     <t xml:space="preserve">[RRAO_RW]  Risk weights (MAR23.8)</t>
   </si>
   <si>
-    <t xml:space="preserve">MAR23.8(1): exotic underlying</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MAR23.8(2): other residual risks</t>
+    <t xml:space="preserve">MAR23.8(2)(a): exotic underlying</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MAR23.8(2)(b): other residual risks</t>
   </si>
   <si>
     <t xml:space="preserve">Regression tests</t>

</xml_diff>

<commit_message>
docs: document the curvature input contract and the covered-bond override limit (#141)
The owner decided on October 27, 2026 (#29, items 2 and 6) to keep two behaviors and document them. A new methodology section states the curvature input contract the upstream pricing must follow (shock sizes per MAR21.98 and MAR21.99, delta deduction, loss-positive sign, one row per risk factor, entry before the FX divisor, no position on sqrt(2) for curvature shocks). A P_CSR override of the covered-bond weight applies to the whole bucket. Interpretation items 2 and 6, the In_Curvature and P_CSR descriptions and the CHANGELOG follow; no calculation changed.

Validated: full suite with LibreOffice and PowerShell (190 passed, 29 subtests), repository checks, CI green, Codex review with no findings. Not validated: desktop Excel (#28).

Resolves #140
</commit_message>
<xml_diff>
--- a/src/workbook/FRTB_Template.xlsx
+++ b/src/workbook/FRTB_Template.xlsx
@@ -688,7 +688,7 @@
     <t xml:space="preserve">Curvature sensitivities</t>
   </si>
   <si>
-    <t xml:space="preserve">Curvature risk CVR up and CVR down per risk factor, net across instruments (MAR21.5(2)).</t>
+    <t xml:space="preserve">Curvature risk CVR up and CVR down per risk factor, net across instruments, positive for a loss and before the FX divisor; shocks per MAR21.98-99 (MAR21.5).</t>
   </si>
   <si>
     <t xml:space="preserve">CVR up</t>
@@ -1174,7 +1174,7 @@
     <t xml:space="preserve">Health care, utilities, professional and technical activities</t>
   </si>
   <si>
-    <t xml:space="preserve">Covered bonds (1.5% for AA- or better at the bank's discretion, fn 17: not modeled)</t>
+    <t xml:space="preserve">Covered bonds (1.5% for AA- or better at the bank's discretion, fn 17: not modeled; an override applies to the whole bucket)</t>
   </si>
   <si>
     <t xml:space="preserve">HY</t>

</xml_diff>